<commit_message>
bom and parts updated
</commit_message>
<xml_diff>
--- a/GaN_Inverter/Project Outputs for GanInverter/Rev02/BOM/BOM_GanInverter_Inverter_V1_Rev02.xlsx
+++ b/GaN_Inverter/Project Outputs for GanInverter/Rev02/BOM/BOM_GanInverter_Inverter_V1_Rev02.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Zeynep\Desktop\Zeynep\software\plugins\github\uz_d_gan_inverter_epc\GaN_Inverter\Project Outputs for GanInverter\Rev02\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{92C819A0-F2DF-483F-BF33-B77A1E3F334D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{13C3F29E-1287-4B65-80EA-ED6C116134D7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="10035" xr2:uid="{50CA122F-30CD-4866-A813-436362A2120C}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="21576" windowHeight="9636" xr2:uid="{A024E7CE-E048-42ED-8118-8E670B7E8557}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_GanInverter_Inverter_V1_Rev" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="555" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="551" uniqueCount="266">
   <si>
     <t>Designator</t>
   </si>
@@ -90,7 +90,7 @@
     <t>1 µF</t>
   </si>
   <si>
-    <t>C2, C3, C7A, C7B, C7C, C8A, C8B, C8C, C9A, C9B, C9C, C10A, C10B, C10C, C11A, C11B, C11C, C12A, C12B, C12C, C13A, C13B, C13C, C14A, C14B, C14C, C19A, C19B, C19C, C24A, C24B, C24C, C26A, C26B, C26C, C28A, C28B, C28C, C31A, C31B, C31C, C36A, C36B, C36C, C46A, C46B, C46C, C47A, C47B, C47C, C48A, C48B, C48C, C49A, C49B, C49C, C50A, C50B, C50C, C51A, C51B, C51C, C52A, C52B, C52C, C53, C54, C55, C56, C61, C64, C89A, C89B, C89C, C90</t>
+    <t>C2, C3, C7A, C7B, C7C, C8A, C8B, C8C, C9A, C9B, C9C, C10A, C10B, C10C, C11A, C11B, C11C, C12A, C12B, C12C, C13A, C13B, C13C, C14A, C14B, C14C, C19A, C19B, C19C, C24A, C24B, C24C, C26A, C26B, C26C, C28A, C28B, C28C, C31A, C31B, C31C, C36A, C36B, C36C, C46A, C46B, C46C, C47A, C47B, C47C, C48A, C48B, C48C, C49A, C49B, C49C, C50A, C50B, C50C, C51A, C51B, C51C, C52A, C52B, C52C</t>
   </si>
   <si>
     <t>Capacitor 0603, 100 VDC, 0.1 uF, X7S</t>
@@ -123,13 +123,10 @@
     <t>C5A, C5B, C5C, C6A, C6B, C6C, C22A, C22B, C22C, C65</t>
   </si>
   <si>
-    <t>Capacitor 0603, 25 VDC, 10 nF, C0G</t>
-  </si>
-  <si>
-    <t>80-C0603X103K3GEC</t>
-  </si>
-  <si>
-    <t>10 nF</t>
+    <t>50V 10nF 2X1 ±10%</t>
+  </si>
+  <si>
+    <t>10nF</t>
   </si>
   <si>
     <t>C15A, C15B, C15C, C16A, C16B, C16C, C17A, C17B, C17C, C57, C59, C60</t>
@@ -147,10 +144,10 @@
     <t>C18A, C18B, C18C, C58</t>
   </si>
   <si>
-    <t>Capacitor 0603, 25 VDC, 0.01 µF, C0G</t>
-  </si>
-  <si>
-    <t>80-C0603C103F3GEC</t>
+    <t>25V 10nF C0G ±5% 0603 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
+  </si>
+  <si>
+    <t>810-C1608C0G1E103J</t>
   </si>
   <si>
     <t>0.01 µF</t>
@@ -159,19 +156,22 @@
     <t>C20A, C20B, C20C, C21</t>
   </si>
   <si>
-    <t>Capacitor 0805, 100 VDC, 0.01 µF, C0G</t>
-  </si>
-  <si>
-    <t>80-C0805C103F1GECAUT</t>
-  </si>
-  <si>
-    <t>C25A, C25B, C25C, C27A, C27B, C27C, C29A, C29B, C29C, C30A, C30B, C30C</t>
-  </si>
-  <si>
-    <t>Capacitor 0805, 50 VDC, 4.7 µF, X7R</t>
-  </si>
-  <si>
-    <t xml:space="preserve">810-C2012X7R475K125C </t>
+    <t>100V 10nF 0805 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
+  </si>
+  <si>
+    <t>HV0805X7R103K101NT</t>
+  </si>
+  <si>
+    <t>JLCPCB</t>
+  </si>
+  <si>
+    <t>C25A, C25B, C25C, C27A, C27B, C27C, C29A, C29B, C29C, C30A, C30B, C30C, C44A, C44B, C44C, C45A, C45B, C45C</t>
+  </si>
+  <si>
+    <t>Capacitor 0603, 35 VDC, 4.7 µF, X5R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">81-GRM188R6YA475KE5D </t>
   </si>
   <si>
     <t>4.7 µF</t>
@@ -192,22 +192,25 @@
     <t>C37A, C37B, C37C, C38A, C38B, C38C, C43A, C43B, C43C</t>
   </si>
   <si>
-    <t>Capacitor 0603, 50 VDC, 22 pF, X7R</t>
-  </si>
-  <si>
-    <t xml:space="preserve">80-C0603C220J5R </t>
+    <t>50V 22pF NP0 ±1% 0603 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
+  </si>
+  <si>
+    <t>603-AC0603FRNP9BN220</t>
   </si>
   <si>
     <t>22 pF</t>
   </si>
   <si>
-    <t>C44A, C44B, C44C, C45A, C45B, C45C</t>
-  </si>
-  <si>
-    <t>Capacitor 0603, 35 VDC, 4.7 µF, X5R</t>
-  </si>
-  <si>
-    <t xml:space="preserve">81-GRM188R6YA475KE5D </t>
+    <t>C53, C54, C55, C56, C61, C64, C89A, C89B, C89C, C90</t>
+  </si>
+  <si>
+    <t>Capacitor 0603, 50 VDC, 100 nF, X7R</t>
+  </si>
+  <si>
+    <t>603-CC603KRX7R9BB104</t>
+  </si>
+  <si>
+    <t>100 nF</t>
   </si>
   <si>
     <t>C67, C68, C70, C72, C74, C76, C78, C80, C82, C84, C86, C88</t>
@@ -240,13 +243,7 @@
     <t>D1</t>
   </si>
   <si>
-    <t>WL-SMCW SMD Mono-color Chip LED Waterclear Blue</t>
-  </si>
-  <si>
-    <t>710-150060BS84000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3408611 </t>
+    <t>LED YELLOW 585.5~591.5NM 90~180MCD@20MA TOP VIEW 0603 ROHS</t>
   </si>
   <si>
     <t>=Manufacturer Part Number</t>
@@ -255,31 +252,25 @@
     <t>WL-SMCW_0603</t>
   </si>
   <si>
+    <t>D2</t>
+  </si>
+  <si>
+    <t>WL-SMCW SMD Mono-color Chip LED Waterclear Red</t>
+  </si>
+  <si>
+    <t xml:space="preserve">710-150060RS86000 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">3408608 </t>
+  </si>
+  <si>
     <t>Farnell</t>
   </si>
   <si>
-    <t>D2</t>
-  </si>
-  <si>
-    <t>WL-SMCW SMD Mono-color Chip LED Waterclear Red</t>
-  </si>
-  <si>
-    <t xml:space="preserve">710-150060RS86000 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">3408608 </t>
-  </si>
-  <si>
     <t>D3</t>
   </si>
   <si>
-    <t>WL-SMCW SMD Mono-color Chip LED Waterclear Green</t>
-  </si>
-  <si>
-    <t>710-150060GS84000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3408612 </t>
+    <t>LED ORANGE 600~610NM 80~220MCD@20MA TOP VIEW 0603 ROHS</t>
   </si>
   <si>
     <t>D4A, D4B, D4C, D5A, D5B, D5C</t>
@@ -456,7 +447,7 @@
     <t>R6</t>
   </si>
   <si>
-    <t>660-RK73B1JTTDD242J</t>
+    <t>100mW ±100ppm/℃ ±1% 2.4kΩ 0603 Chip Resistor - Surface Mount ROHS</t>
   </si>
   <si>
     <t>2k4</t>
@@ -465,7 +456,7 @@
     <t>R7</t>
   </si>
   <si>
-    <t>660-RK73B1JTTDD682J</t>
+    <t>100mW ±100ppm/℃ ±5% 6.8kΩ 0603  Chip Resistor - Surface Mount ROHS</t>
   </si>
   <si>
     <t>6k8</t>
@@ -510,7 +501,7 @@
     <t>R24A, R24B, R24C, R25A, R25B, R25C</t>
   </si>
   <si>
-    <t>652-CR0603-FX1053ELF</t>
+    <t>100mW Thick Film Resistors ±100ppm/℃ ±1% 105kΩ 0603 Chip Resistor - Surface Mount ROHS</t>
   </si>
   <si>
     <t>105k</t>
@@ -519,7 +510,7 @@
     <t>R26A, R26B, R26C, R27A, R27B, R27C</t>
   </si>
   <si>
-    <t>652-CR0603-FX2803ELF</t>
+    <t>100mW Thin Film Resistor ±50ppm/℃ ±0.1% 280kΩ 0603 Chip Resistor - Surface Mount ROHS</t>
   </si>
   <si>
     <t>280k</t>
@@ -558,7 +549,7 @@
     <t>R35A, R35B, R35C, R36A, R36B, R36C, R41A, R41B, R41C, R46A, R46B, R46C, R74, R78, R82, R87</t>
   </si>
   <si>
-    <t>279-RQ73C1J110KBTD</t>
+    <t>100mW Thick Film Resistors ±100ppm/℃ ±1% 110kΩ 0603 Chip Resistor - Surface Mount ROHS</t>
   </si>
   <si>
     <t>110k</t>
@@ -567,7 +558,10 @@
     <t>R38A, R38B, R38C, R39A, R39B, R39C, R48A, R48B, R48C, R79, R80, R89</t>
   </si>
   <si>
-    <t>66-PCFW0603LF031001B</t>
+    <t>SMD resistor E24 series 470 kOhms 100-200 mW 0603 1%</t>
+  </si>
+  <si>
+    <t>LCSC/JLCPCB</t>
   </si>
   <si>
     <t>1k</t>
@@ -600,7 +594,7 @@
     <t>R49A, R49B, R49C, R50A, R50B, R50C</t>
   </si>
   <si>
-    <t>660-RK73B1JTTDD221J</t>
+    <t>125mW ±100ppm/℃ ±5% 220Ω 0603 Chip Resistor - Surface Mount ROHS</t>
   </si>
   <si>
     <t>220R</t>
@@ -609,7 +603,7 @@
     <t>R53A, R53B, R53C, R54A, R54B, R54C</t>
   </si>
   <si>
-    <t xml:space="preserve">71-CRCW0603100KFKEAC </t>
+    <t>100mW Thick Film Resistors ±100ppm/℃ ±1% 100kΩ 0603 Chip Resistor - Surface Mount ROHS</t>
   </si>
   <si>
     <t>100k</t>
@@ -828,10 +822,7 @@
     <t>Pin Header 3x2</t>
   </si>
   <si>
-    <t>200-TSW10305GDLL</t>
-  </si>
-  <si>
-    <t>Pin Header</t>
+    <t>ZHOURI 2.54-1*3</t>
   </si>
   <si>
     <t>SAMTEC_TSW-103-05-G-D</t>
@@ -1210,18 +1201,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF127F9D-A8BB-46BF-8512-2370360F2C99}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0DBD9C68-4D86-4CB3-A06A-989B7B68AEA4}">
   <dimension ref="A1:K62"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.42578125" customWidth="1"/>
-    <col min="2" max="2" width="12.7109375" customWidth="1"/>
-    <col min="3" max="3" width="59.5703125" customWidth="1"/>
-    <col min="4" max="4" width="9.28515625" customWidth="1"/>
-    <col min="5" max="11" width="16.5703125" customWidth="1"/>
+    <col min="1" max="1" width="16.88671875" customWidth="1"/>
+    <col min="2" max="2" width="12.33203125" customWidth="1"/>
+    <col min="3" max="3" width="57.33203125" customWidth="1"/>
+    <col min="4" max="4" width="9" customWidth="1"/>
+    <col min="5" max="11" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1256,7 +1247,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>11</v>
       </c>
@@ -1289,7 +1280,7 @@
       </c>
       <c r="K2" s="1"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>20</v>
       </c>
@@ -1309,7 +1300,7 @@
         <v>16</v>
       </c>
       <c r="G3" s="1">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>18</v>
@@ -1322,7 +1313,7 @@
       </c>
       <c r="K3" s="1"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>25</v>
       </c>
@@ -1355,7 +1346,7 @@
       </c>
       <c r="K4" s="1"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>30</v>
       </c>
@@ -1363,13 +1354,13 @@
         <v>31</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>23</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>16</v>
@@ -1378,25 +1369,25 @@
         <v>10</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>23</v>
       </c>
       <c r="J5" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="K5" s="1"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="K5" s="1"/>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
+      <c r="B6" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="2" t="s">
         <v>35</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>36</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>13</v>
@@ -1417,19 +1408,19 @@
         <v>17</v>
       </c>
       <c r="J6" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="K6" s="1"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="K6" s="1"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
+      <c r="B7" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="C7" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>40</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>23</v>
@@ -1450,19 +1441,19 @@
         <v>23</v>
       </c>
       <c r="J7" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="K7" s="1"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="K7" s="1"/>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
+      <c r="B8" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="C8" s="2" t="s">
         <v>43</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>44</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>23</v>
@@ -1477,17 +1468,17 @@
         <v>4</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>23</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K8" s="1"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>45</v>
       </c>
@@ -1504,10 +1495,10 @@
         <v>15</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="G9" s="1">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H9" s="2" t="s">
         <v>18</v>
@@ -1520,7 +1511,7 @@
       </c>
       <c r="K9" s="1"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>49</v>
       </c>
@@ -1553,7 +1544,7 @@
       </c>
       <c r="K10" s="1"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>53</v>
       </c>
@@ -1586,7 +1577,7 @@
       </c>
       <c r="K11" s="1"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>57</v>
       </c>
@@ -1594,10 +1585,10 @@
         <v>58</v>
       </c>
       <c r="C12" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>59</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>23</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>15</v>
@@ -1606,28 +1597,28 @@
         <v>16</v>
       </c>
       <c r="G12" s="1">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="K12" s="1"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>23</v>
@@ -1636,7 +1627,7 @@
         <v>15</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G13" s="1">
         <v>12</v>
@@ -1652,15 +1643,15 @@
       </c>
       <c r="K13" s="1"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>23</v>
@@ -1669,7 +1660,7 @@
         <v>15</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G14" s="1">
         <v>10</v>
@@ -1681,59 +1672,55 @@
         <v>23</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="K14" s="1"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="D15" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" s="1"/>
+      <c r="E15" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="E15" s="2" t="s">
+      <c r="F15" s="2" t="s">
         <v>73</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>74</v>
       </c>
       <c r="G15" s="1">
         <v>1</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="I15" s="2" t="s">
-        <v>75</v>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="I15" s="1"/>
       <c r="J15" s="1"/>
       <c r="K15" s="1"/>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="D16" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>79</v>
-      </c>
       <c r="E16" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F16" s="2" t="s">
         <v>73</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>74</v>
       </c>
       <c r="G16" s="1">
         <v>1</v>
@@ -1742,60 +1729,56 @@
         <v>18</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="J16" s="1"/>
       <c r="K16" s="1"/>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="B17" s="2" t="s">
-        <v>81</v>
-      </c>
       <c r="C17" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>83</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="D17" s="1"/>
       <c r="E17" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F17" s="2" t="s">
         <v>73</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>74</v>
       </c>
       <c r="G17" s="1">
         <v>1</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="I17" s="2" t="s">
-        <v>75</v>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="I17" s="1"/>
       <c r="J17" s="1"/>
       <c r="K17" s="1"/>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F18" s="2" t="s">
         <v>84</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>87</v>
       </c>
       <c r="G18" s="1">
         <v>6</v>
@@ -1811,24 +1794,24 @@
       </c>
       <c r="K18" s="1"/>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F19" s="2" t="s">
         <v>88</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>91</v>
       </c>
       <c r="G19" s="1">
         <v>3</v>
@@ -1840,16 +1823,16 @@
         <v>23</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="K19" s="1"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>13</v>
@@ -1858,10 +1841,10 @@
         <v>23</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="G20" s="1">
         <v>2</v>
@@ -1877,123 +1860,123 @@
       </c>
       <c r="K20" s="1"/>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="D21" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="E21" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="F21" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>101</v>
       </c>
       <c r="G21" s="1">
         <v>3</v>
       </c>
       <c r="H21" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="J21" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="K21" s="1"/>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A22" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="I21" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="J21" s="2" t="s">
+      <c r="C22" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="K21" s="1"/>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A22" s="2" t="s">
+      <c r="D22" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="E22" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="C22" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>108</v>
-      </c>
       <c r="F22" s="2" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="G22" s="1">
         <v>1</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="J22" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="K22" s="1"/>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A23" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="K22" s="1"/>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A23" s="2" t="s">
+      <c r="D23" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="E23" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="C23" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>114</v>
-      </c>
       <c r="F23" s="2" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="G23" s="1">
         <v>1</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="J23" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="K23" s="1"/>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A24" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="K23" s="1"/>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A24" s="2" t="s">
+      <c r="D24" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F24" s="2" t="s">
         <v>116</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>119</v>
       </c>
       <c r="G24" s="1">
         <v>8</v>
@@ -2009,24 +1992,24 @@
       </c>
       <c r="K24" s="1"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="D25" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="E25" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F25" s="2" t="s">
         <v>121</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>124</v>
       </c>
       <c r="G25" s="1">
         <v>25</v>
@@ -2035,19 +2018,19 @@
         <v>18</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="J25" s="2" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="K25" s="1"/>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>13</v>
@@ -2056,10 +2039,10 @@
         <v>23</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="G26" s="1">
         <v>6</v>
@@ -2068,22 +2051,22 @@
         <v>17</v>
       </c>
       <c r="I26" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="J26" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="K26" s="1"/>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A27" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B27" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="J26" s="2" t="s">
+      <c r="C27" s="2" t="s">
         <v>130</v>
-      </c>
-      <c r="K26" s="1"/>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A27" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>133</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>13</v>
@@ -2092,7 +2075,7 @@
         <v>15</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="G27" s="1">
         <v>20</v>
@@ -2104,19 +2087,19 @@
         <v>17</v>
       </c>
       <c r="J27" s="2" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="K27" s="1"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>23</v>
@@ -2125,7 +2108,7 @@
         <v>15</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="G28" s="1">
         <v>25</v>
@@ -2137,16 +2120,16 @@
         <v>23</v>
       </c>
       <c r="J28" s="2" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="K28" s="1"/>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>13</v>
@@ -2158,7 +2141,7 @@
         <v>15</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="G29" s="1">
         <v>7</v>
@@ -2170,86 +2153,86 @@
         <v>23</v>
       </c>
       <c r="J29" s="2" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="K29" s="1"/>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>142</v>
+        <v>13</v>
       </c>
       <c r="D30" s="1"/>
       <c r="E30" s="2" t="s">
         <v>15</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="G30" s="1">
         <v>1</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I30" s="1"/>
       <c r="J30" s="2" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="K30" s="1"/>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>145</v>
+        <v>13</v>
       </c>
       <c r="D31" s="1"/>
       <c r="E31" s="2" t="s">
         <v>15</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="G31" s="1">
         <v>1</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I31" s="1"/>
       <c r="J31" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="K31" s="1"/>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A32" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="C32" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="K31" s="1"/>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A32" s="2" t="s">
+      <c r="D32" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F32" s="2" t="s">
         <v>147</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>148</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E32" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F32" s="2" t="s">
-        <v>150</v>
       </c>
       <c r="G32" s="1">
         <v>6</v>
@@ -2261,20 +2244,20 @@
         <v>23</v>
       </c>
       <c r="J32" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="K32" s="1"/>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A33" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="C33" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="K32" s="1"/>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A33" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>154</v>
-      </c>
       <c r="D33" s="2" t="s">
         <v>23</v>
       </c>
@@ -2282,7 +2265,7 @@
         <v>15</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="G33" s="1">
         <v>6</v>
@@ -2294,19 +2277,19 @@
         <v>23</v>
       </c>
       <c r="J33" s="2" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="K33" s="1"/>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>23</v>
@@ -2315,7 +2298,7 @@
         <v>15</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="G34" s="1">
         <v>6</v>
@@ -2327,19 +2310,19 @@
         <v>23</v>
       </c>
       <c r="J34" s="2" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="K34" s="1"/>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>160</v>
+        <v>13</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>23</v>
@@ -2348,31 +2331,31 @@
         <v>15</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="G35" s="1">
         <v>6</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I35" s="2" t="s">
         <v>23</v>
       </c>
       <c r="J35" s="2" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="K35" s="1"/>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>163</v>
+        <v>13</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>23</v>
@@ -2381,31 +2364,31 @@
         <v>15</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="G36" s="1">
         <v>6</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I36" s="2" t="s">
         <v>23</v>
       </c>
       <c r="J36" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="K36" s="1"/>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>13</v>
@@ -2414,7 +2397,7 @@
         <v>15</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="G37" s="1">
         <v>16</v>
@@ -2426,19 +2409,19 @@
         <v>17</v>
       </c>
       <c r="J37" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="K37" s="1"/>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A38" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="C38" s="2" t="s">
         <v>167</v>
-      </c>
-      <c r="K37" s="1"/>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A38" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>170</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>13</v>
@@ -2447,7 +2430,7 @@
         <v>15</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="G38" s="1">
         <v>12</v>
@@ -2459,20 +2442,20 @@
         <v>17</v>
       </c>
       <c r="J38" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="K38" s="1"/>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A39" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="C39" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="K38" s="1"/>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A39" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>174</v>
-      </c>
       <c r="D39" s="2" t="s">
         <v>23</v>
       </c>
@@ -2480,7 +2463,7 @@
         <v>15</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="G39" s="1">
         <v>16</v>
@@ -2492,19 +2475,19 @@
         <v>23</v>
       </c>
       <c r="J39" s="2" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="K39" s="1"/>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>173</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>176</v>
+        <v>13</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>23</v>
@@ -2513,31 +2496,31 @@
         <v>15</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="G40" s="1">
         <v>16</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I40" s="2" t="s">
         <v>23</v>
       </c>
       <c r="J40" s="2" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="K40" s="1"/>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>179</v>
+        <v>13</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>23</v>
@@ -2546,32 +2529,32 @@
         <v>15</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="G41" s="1">
         <v>12</v>
       </c>
       <c r="H41" s="2" t="s">
-        <v>18</v>
+        <v>177</v>
       </c>
       <c r="I41" s="2" t="s">
         <v>23</v>
       </c>
       <c r="J41" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="K41" s="1"/>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A42" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="C42" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="K41" s="1"/>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A42" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="B42" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>182</v>
-      </c>
       <c r="D42" s="2" t="s">
         <v>23</v>
       </c>
@@ -2579,7 +2562,7 @@
         <v>15</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="G42" s="1">
         <v>8</v>
@@ -2591,28 +2574,28 @@
         <v>23</v>
       </c>
       <c r="J42" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="K42" s="1"/>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A43" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B43" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="K42" s="1"/>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A43" s="2" t="s">
+      <c r="C43" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="B43" s="2" t="s">
+      <c r="D43" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F43" s="2" t="s">
         <v>185</v>
-      </c>
-      <c r="C43" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="D43" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E43" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F43" s="2" t="s">
-        <v>187</v>
       </c>
       <c r="G43" s="1">
         <v>4</v>
@@ -2624,19 +2607,19 @@
         <v>23</v>
       </c>
       <c r="J43" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="K43" s="1"/>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A44" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="B44" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="K43" s="1"/>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A44" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="B44" s="2" t="s">
-        <v>132</v>
-      </c>
       <c r="C44" s="2" t="s">
-        <v>190</v>
+        <v>13</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>23</v>
@@ -2645,31 +2628,31 @@
         <v>15</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="G44" s="1">
         <v>6</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I44" s="2" t="s">
         <v>23</v>
       </c>
       <c r="J44" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="K44" s="1"/>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A45" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="B45" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="K44" s="1"/>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A45" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>148</v>
-      </c>
       <c r="C45" s="2" t="s">
-        <v>193</v>
+        <v>13</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>23</v>
@@ -2678,61 +2661,61 @@
         <v>15</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="G45" s="1">
         <v>6</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I45" s="2" t="s">
         <v>23</v>
       </c>
       <c r="J45" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="K45" s="1"/>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A46" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="C46" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="K45" s="1"/>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A46" s="2" t="s">
+      <c r="D46" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F46" s="2" t="s">
         <v>195</v>
-      </c>
-      <c r="B46" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="C46" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="D46" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E46" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F46" s="2" t="s">
-        <v>197</v>
       </c>
       <c r="G46" s="1">
         <v>6</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="I46" s="2" t="s">
         <v>23</v>
       </c>
       <c r="J46" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="K46" s="1"/>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A47" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="B47" s="2" t="s">
         <v>198</v>
-      </c>
-      <c r="K46" s="1"/>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A47" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="B47" s="2" t="s">
-        <v>200</v>
       </c>
       <c r="C47" s="2" t="s">
         <v>13</v>
@@ -2744,7 +2727,7 @@
         <v>15</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="G47" s="1">
         <v>12</v>
@@ -2756,16 +2739,16 @@
         <v>23</v>
       </c>
       <c r="J47" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="K47" s="1"/>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A48" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="B48" s="2" t="s">
         <v>201</v>
-      </c>
-      <c r="K47" s="1"/>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A48" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="B48" s="2" t="s">
-        <v>203</v>
       </c>
       <c r="C48" s="2" t="s">
         <v>13</v>
@@ -2777,7 +2760,7 @@
         <v>15</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="G48" s="1">
         <v>3</v>
@@ -2789,16 +2772,16 @@
         <v>23</v>
       </c>
       <c r="J48" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="K48" s="1"/>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A49" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="B49" s="2" t="s">
         <v>204</v>
-      </c>
-      <c r="K48" s="1"/>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A49" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="B49" s="2" t="s">
-        <v>206</v>
       </c>
       <c r="C49" s="2" t="s">
         <v>13</v>
@@ -2810,7 +2793,7 @@
         <v>15</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="G49" s="1">
         <v>6</v>
@@ -2822,16 +2805,16 @@
         <v>23</v>
       </c>
       <c r="J49" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="K49" s="1"/>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A50" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="B50" s="2" t="s">
         <v>207</v>
-      </c>
-      <c r="K49" s="1"/>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A50" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="B50" s="2" t="s">
-        <v>209</v>
       </c>
       <c r="C50" s="2" t="s">
         <v>13</v>
@@ -2843,7 +2826,7 @@
         <v>15</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="G50" s="1">
         <v>9</v>
@@ -2855,28 +2838,28 @@
         <v>23</v>
       </c>
       <c r="J50" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="K50" s="1"/>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A51" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="B51" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="K50" s="1"/>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A51" s="2" t="s">
+      <c r="C51" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="B51" s="2" t="s">
+      <c r="D51" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="C51" s="2" t="s">
+      <c r="E51" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F51" s="2" t="s">
         <v>214</v>
-      </c>
-      <c r="D51" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="E51" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="F51" s="2" t="s">
-        <v>216</v>
       </c>
       <c r="G51" s="1">
         <v>1</v>
@@ -2885,31 +2868,31 @@
         <v>18</v>
       </c>
       <c r="I51" s="2" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="J51" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="K51" s="1"/>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A52" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="B52" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="K51" s="1"/>
-    </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A52" s="2" t="s">
+      <c r="C52" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="B52" s="2" t="s">
+      <c r="D52" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F52" s="2" t="s">
         <v>219</v>
-      </c>
-      <c r="C52" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="D52" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E52" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="F52" s="2" t="s">
-        <v>221</v>
       </c>
       <c r="G52" s="1">
         <v>6</v>
@@ -2925,24 +2908,24 @@
       </c>
       <c r="K52" s="1"/>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="C53" s="2" t="s">
         <v>222</v>
       </c>
-      <c r="B53" s="2" t="s">
+      <c r="D53" s="2" t="s">
         <v>223</v>
       </c>
-      <c r="C53" s="2" t="s">
+      <c r="E53" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F53" s="2" t="s">
         <v>224</v>
-      </c>
-      <c r="D53" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="E53" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="F53" s="2" t="s">
-        <v>226</v>
       </c>
       <c r="G53" s="1">
         <v>8</v>
@@ -2951,31 +2934,31 @@
         <v>18</v>
       </c>
       <c r="I53" s="2" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="J53" s="2" t="s">
         <v>23</v>
       </c>
       <c r="K53" s="1"/>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="C54" s="2" t="s">
         <v>227</v>
       </c>
-      <c r="B54" s="2" t="s">
+      <c r="D54" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="C54" s="2" t="s">
+      <c r="E54" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F54" s="2" t="s">
         <v>229</v>
-      </c>
-      <c r="D54" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="E54" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="F54" s="2" t="s">
-        <v>231</v>
       </c>
       <c r="G54" s="1">
         <v>6</v>
@@ -2984,31 +2967,31 @@
         <v>18</v>
       </c>
       <c r="I54" s="2" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="J54" s="2" t="s">
         <v>23</v>
       </c>
       <c r="K54" s="1"/>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="C55" s="2" t="s">
         <v>232</v>
       </c>
-      <c r="B55" s="2" t="s">
+      <c r="D55" s="2" t="s">
         <v>233</v>
       </c>
-      <c r="C55" s="2" t="s">
+      <c r="E55" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F55" s="2" t="s">
         <v>234</v>
-      </c>
-      <c r="D55" s="2" t="s">
-        <v>235</v>
-      </c>
-      <c r="E55" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="F55" s="2" t="s">
-        <v>236</v>
       </c>
       <c r="G55" s="1">
         <v>6</v>
@@ -3017,31 +3000,31 @@
         <v>18</v>
       </c>
       <c r="I55" s="2" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="J55" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="K55" s="1"/>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A56" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="B56" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="K55" s="1"/>
-    </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A56" s="2" t="s">
+      <c r="C56" s="2" t="s">
         <v>238</v>
       </c>
-      <c r="B56" s="2" t="s">
+      <c r="D56" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E56" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F56" s="2" t="s">
         <v>239</v>
-      </c>
-      <c r="C56" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="D56" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E56" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="F56" s="2" t="s">
-        <v>241</v>
       </c>
       <c r="G56" s="1">
         <v>4</v>
@@ -3056,27 +3039,27 @@
         <v>23</v>
       </c>
       <c r="K56" s="2" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A57" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="B57" s="2" t="s">
         <v>242</v>
       </c>
-    </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A57" s="2" t="s">
+      <c r="C57" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="B57" s="2" t="s">
+      <c r="D57" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E57" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F57" s="2" t="s">
         <v>244</v>
-      </c>
-      <c r="C57" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="D57" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E57" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="F57" s="2" t="s">
-        <v>246</v>
       </c>
       <c r="G57" s="1">
         <v>6</v>
@@ -3092,24 +3075,24 @@
       </c>
       <c r="K57" s="1"/>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="C58" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="B58" s="2" t="s">
+      <c r="D58" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E58" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F58" s="2" t="s">
         <v>248</v>
-      </c>
-      <c r="C58" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="D58" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E58" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="F58" s="2" t="s">
-        <v>250</v>
       </c>
       <c r="G58" s="1">
         <v>6</v>
@@ -3125,24 +3108,24 @@
       </c>
       <c r="K58" s="1"/>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="C59" s="2" t="s">
         <v>251</v>
       </c>
-      <c r="B59" s="2" t="s">
+      <c r="D59" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E59" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F59" s="2" t="s">
         <v>252</v>
-      </c>
-      <c r="C59" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="D59" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E59" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="F59" s="2" t="s">
-        <v>254</v>
       </c>
       <c r="G59" s="1">
         <v>3</v>
@@ -3158,24 +3141,24 @@
       </c>
       <c r="K59" s="1"/>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="C60" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="B60" s="2" t="s">
+      <c r="D60" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E60" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F60" s="2" t="s">
         <v>256</v>
-      </c>
-      <c r="C60" s="2" t="s">
-        <v>257</v>
-      </c>
-      <c r="D60" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E60" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F60" s="2" t="s">
-        <v>258</v>
       </c>
       <c r="G60" s="1">
         <v>6</v>
@@ -3187,28 +3170,28 @@
         <v>23</v>
       </c>
       <c r="J60" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="K60" s="1"/>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A61" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="B61" s="2" t="s">
         <v>259</v>
       </c>
-      <c r="K60" s="1"/>
-    </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A61" s="2" t="s">
+      <c r="C61" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="B61" s="2" t="s">
-        <v>261</v>
-      </c>
-      <c r="C61" s="2" t="s">
-        <v>262</v>
-      </c>
       <c r="D61" s="2" t="s">
         <v>23</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="G61" s="1">
         <v>4</v>
@@ -3223,33 +3206,33 @@
         <v>23</v>
       </c>
       <c r="K61" s="2" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A62" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="B62" s="2" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A62" s="2" t="s">
+      <c r="C62" s="2" t="s">
         <v>264</v>
       </c>
-      <c r="B62" s="2" t="s">
+      <c r="D62" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E62" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F62" s="2" t="s">
         <v>265</v>
-      </c>
-      <c r="C62" s="2" t="s">
-        <v>266</v>
-      </c>
-      <c r="D62" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E62" s="2" t="s">
-        <v>267</v>
-      </c>
-      <c r="F62" s="2" t="s">
-        <v>268</v>
       </c>
       <c r="G62" s="1">
         <v>3</v>
       </c>
       <c r="H62" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I62" s="2" t="s">
         <v>23</v>

</xml_diff>

<commit_message>
final BOM including all LCSC part numbers required
</commit_message>
<xml_diff>
--- a/GaN_Inverter/Project Outputs for GanInverter/Rev02/BOM/BOM_GanInverter_Inverter_V1_Rev02.xlsx
+++ b/GaN_Inverter/Project Outputs for GanInverter/Rev02/BOM/BOM_GanInverter_Inverter_V1_Rev02.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Zeynep\Desktop\Zeynep\software\plugins\github\uz_d_gan_inverter_epc\GaN_Inverter\Project Outputs for GanInverter\Rev02\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C0B66306-75D1-44A4-BE6B-69AC4DB97A1D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D1CD8DC1-C8F5-4A53-97C7-DFB7D7B48565}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21576" windowHeight="9636" xr2:uid="{22DE773A-3BCE-4473-B976-9536B773EE11}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="9555" xr2:uid="{4561B4DB-BFCF-43FF-9293-E14FB912EADC}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_GanInverter_Inverter_V1_Rev" sheetId="1" r:id="rId1"/>
@@ -123,7 +123,7 @@
     <t>C32A, C32B, C32C, C33A, C33B, C33C</t>
   </si>
   <si>
-    <t>C2167215</t>
+    <t>C2929194</t>
   </si>
   <si>
     <t>22 pF</t>
@@ -264,7 +264,7 @@
     <t>C3347196</t>
   </si>
   <si>
-    <t>LQM18DN6R8M70L</t>
+    <t>6.8uH</t>
   </si>
   <si>
     <t>L1, L2A, L2B, L2C, L3A, L3B, L3C, L4A, L4B, L4C, L5A, L5B, L5C, L6A, L6B, L6C, L7A, L7B, L7C, L8A, L8B, L8C, L9, L10, L11</t>
@@ -273,7 +273,7 @@
     <t>INDC1608X95N</t>
   </si>
   <si>
-    <t>C1881372</t>
+    <t>C961362</t>
   </si>
   <si>
     <t>EPC2302</t>
@@ -390,7 +390,7 @@
     <t>R28A, R28B, R28C, R29A, R29B, R29C, R30A, R30B, R30C, R31A, R31B, R31C, R69, R70, R71, R72</t>
   </si>
   <si>
-    <t>C160046</t>
+    <t>C2075693</t>
   </si>
   <si>
     <t>2k</t>
@@ -399,7 +399,7 @@
     <t>R32A, R32B, R32C, R33A, R33B, R33C, R43A, R43B, R43C, R73, R76, R84</t>
   </si>
   <si>
-    <t>C189729</t>
+    <t>C705921, C189729</t>
   </si>
   <si>
     <t>110k</t>
@@ -570,7 +570,7 @@
     <t>C6730719</t>
   </si>
   <si>
-    <t>MAX40056TAUA+</t>
+    <t>Value</t>
   </si>
   <si>
     <t>U8A, U8B, U8C, U16</t>
@@ -579,7 +579,7 @@
     <t>SOP65P490X110-8N</t>
   </si>
   <si>
-    <t>C1139026</t>
+    <t>C4550714</t>
   </si>
   <si>
     <t>MAX14931FASE+</t>
@@ -1021,17 +1021,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B627FF04-3AC1-4BEB-9EBF-9046EF541C85}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{002A033D-825E-4A9A-8989-114CA7960F77}">
   <dimension ref="A1:D61"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.44140625" customWidth="1"/>
-    <col min="2" max="2" width="17" customWidth="1"/>
-    <col min="3" max="3" width="23.44140625" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="1" max="1" width="19" customWidth="1"/>
+    <col min="2" max="2" width="17.5703125" customWidth="1"/>
+    <col min="3" max="3" width="24.28515625" customWidth="1"/>
+    <col min="4" max="4" width="16.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1045,7 +1045,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -1059,7 +1059,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
@@ -1073,7 +1073,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
@@ -1087,7 +1087,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>15</v>
       </c>
@@ -1101,7 +1101,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>18</v>
       </c>
@@ -1115,7 +1115,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>21</v>
       </c>
@@ -1129,7 +1129,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>21</v>
       </c>
@@ -1143,7 +1143,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>26</v>
       </c>
@@ -1157,7 +1157,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>29</v>
       </c>
@@ -1171,7 +1171,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>32</v>
       </c>
@@ -1185,7 +1185,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>35</v>
       </c>
@@ -1199,7 +1199,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
@@ -1213,7 +1213,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>41</v>
       </c>
@@ -1227,7 +1227,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>45</v>
       </c>
@@ -1241,7 +1241,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>49</v>
       </c>
@@ -1255,7 +1255,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>52</v>
       </c>
@@ -1269,7 +1269,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>55</v>
       </c>
@@ -1283,7 +1283,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>59</v>
       </c>
@@ -1297,7 +1297,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>63</v>
       </c>
@@ -1311,7 +1311,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>67</v>
       </c>
@@ -1323,7 +1323,7 @@
       </c>
       <c r="D21" s="1"/>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>70</v>
       </c>
@@ -1335,7 +1335,7 @@
       </c>
       <c r="D22" s="1"/>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>72</v>
       </c>
@@ -1347,7 +1347,7 @@
       </c>
       <c r="D23" s="1"/>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>74</v>
       </c>
@@ -1361,7 +1361,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>78</v>
       </c>
@@ -1375,7 +1375,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>82</v>
       </c>
@@ -1389,7 +1389,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>86</v>
       </c>
@@ -1403,7 +1403,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>90</v>
       </c>
@@ -1417,7 +1417,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>93</v>
       </c>
@@ -1431,7 +1431,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>96</v>
       </c>
@@ -1445,7 +1445,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>99</v>
       </c>
@@ -1459,7 +1459,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>102</v>
       </c>
@@ -1473,7 +1473,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>106</v>
       </c>
@@ -1487,7 +1487,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>109</v>
       </c>
@@ -1501,7 +1501,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>112</v>
       </c>
@@ -1515,7 +1515,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>115</v>
       </c>
@@ -1529,7 +1529,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>118</v>
       </c>
@@ -1543,7 +1543,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>121</v>
       </c>
@@ -1557,7 +1557,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>124</v>
       </c>
@@ -1571,7 +1571,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>127</v>
       </c>
@@ -1585,7 +1585,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>130</v>
       </c>
@@ -1599,7 +1599,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>133</v>
       </c>
@@ -1613,7 +1613,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>137</v>
       </c>
@@ -1627,7 +1627,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>140</v>
       </c>
@@ -1641,7 +1641,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>143</v>
       </c>
@@ -1655,7 +1655,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>147</v>
       </c>
@@ -1669,7 +1669,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>150</v>
       </c>
@@ -1683,7 +1683,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>153</v>
       </c>
@@ -1697,7 +1697,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>156</v>
       </c>
@@ -1711,7 +1711,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>160</v>
       </c>
@@ -1725,7 +1725,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>164</v>
       </c>
@@ -1739,7 +1739,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>168</v>
       </c>
@@ -1753,7 +1753,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>172</v>
       </c>
@@ -1767,7 +1767,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>176</v>
       </c>
@@ -1781,7 +1781,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
         <v>180</v>
       </c>
@@ -1795,7 +1795,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>184</v>
       </c>
@@ -1809,7 +1809,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>188</v>
       </c>
@@ -1823,7 +1823,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
         <v>191</v>
       </c>
@@ -1837,7 +1837,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
         <v>195</v>
       </c>
@@ -1851,7 +1851,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
         <v>199</v>
       </c>
@@ -1865,7 +1865,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
         <v>202</v>
       </c>

</xml_diff>